<commit_message>
Add Al-electrode sweep results to raw-data spreadsheet
Al bottom electrode (material.l_Al_JO), ETL/HTL 500 nm, both substrates:
- n=1.51: planar 0.179, EQE_sub 0.480, SL 0.228-0.370
- n=1.80: planar 0.178, EQE_sub 0.777, SL up to 0.540
Al absorption weakens the recycling, so EQE is lower than with Ag and
the S-g dependence is stronger at large S(1-g).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -10,10 +10,12 @@
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="n1.80_ETLHTL500" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="n1.51_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="n1.80_ETLHTL80" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="n1.51_ETLHTL80" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="n1.51_ETLHTL150" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="n1.51_ETLHTL200" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="n1.80_ETLHTL500_Al" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="n1.51_ETLHTL500_Al" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="n1.80_ETLHTL80" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.51_ETLHTL80" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="n1.51_ETLHTL150" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="n1.51_ETLHTL200" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -578,72 +580,108 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL80</t>
+          <t>n1.80_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.1854</v>
+        <v>0.1778</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.7775</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL80</t>
+          <t>n1.51_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.1794</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.5525</v>
+        <v>0.4801</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL150</t>
+          <t>n1.80_ETLHTL80</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.1311</v>
+        <v>0.1854</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.8097</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>n1.51_ETLHTL80</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0.1865</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>0.5525</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>n1.51_ETLHTL150</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>0.1311</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>0.4005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>n1.51_ETLHTL200</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C16" s="2" t="n">
         <v>0.3347</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D16" s="2" t="n">
         <v>0.5671</v>
       </c>
     </row>
@@ -1191,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1201,12 +1239,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -1232,6 +1271,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1240,22 +1282,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.721296</v>
+        <v>0.527973</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.720206</v>
+        <v>0.527058</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.716857</v>
+        <v>0.522398</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.707013</v>
+        <v>0.508132</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.672125</v>
+        <v>0.464831</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.182393</v>
+        <v>0.401885</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.176671</v>
       </c>
     </row>
     <row r="5">
@@ -1263,22 +1308,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.716266</v>
+        <v>0.513765</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.721016</v>
+        <v>0.523353</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.725425</v>
+        <v>0.533013</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.728177</v>
+        <v>0.539902</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.723059</v>
+        <v>0.53354</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.182389</v>
+        <v>0.5025810000000001</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.176663</v>
       </c>
     </row>
     <row r="6">
@@ -1286,22 +1334,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.698484</v>
+        <v>0.481836</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.707616</v>
+        <v>0.497634</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.716408</v>
+        <v>0.5140169999999999</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.724815</v>
+        <v>0.531281</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.72904</v>
+        <v>0.542503</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.182388</v>
+        <v>0.529126</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.176665</v>
       </c>
     </row>
     <row r="7">
@@ -1309,22 +1360,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6793630000000001</v>
+        <v>0.452262</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.692587</v>
+        <v>0.472202</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.705593</v>
+        <v>0.494101</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.718198</v>
+        <v>0.517697</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.728581</v>
+        <v>0.5401</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.182403</v>
+        <v>0.539558</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.176684</v>
       </c>
     </row>
     <row r="8">
@@ -1332,22 +1386,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.660434</v>
+        <v>0.426585</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.677283</v>
+        <v>0.4493</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.694479</v>
+        <v>0.475345</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.7111769999999999</v>
+        <v>0.504194</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.726436</v>
+        <v>0.534932</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.182386</v>
+        <v>0.5428269999999999</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.176655</v>
       </c>
     </row>
     <row r="9">
@@ -1355,22 +1412,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.64097</v>
+        <v>0.402791</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.662505</v>
+        <v>0.429294</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.6832780000000001</v>
+        <v>0.458065</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.703989</v>
+        <v>0.491371</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.723368</v>
+        <v>0.528176</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.182387</v>
+        <v>0.5435759999999999</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.176657</v>
       </c>
     </row>
     <row r="10">
@@ -1378,22 +1438,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.622152</v>
+        <v>0.381897</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6469510000000001</v>
+        <v>0.409937</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671573</v>
+        <v>0.441454</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.696204</v>
+        <v>0.478134</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.719983</v>
+        <v>0.521226</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.182385</v>
+        <v>0.541695</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.176651</v>
       </c>
     </row>
     <row r="11">
@@ -1401,22 +1464,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.604131</v>
+        <v>0.363437</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.631347</v>
+        <v>0.391913</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.659758</v>
+        <v>0.425692</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.68865</v>
+        <v>0.466244</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.716566</v>
+        <v>0.514435</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.182391</v>
+        <v>0.53949</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.176667</v>
       </c>
     </row>
   </sheetData>
@@ -1430,7 +1496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1440,12 +1506,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -1471,6 +1538,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1479,22 +1549,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.51635</v>
+        <v>0.364003</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.516308</v>
+        <v>0.364627</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.515298</v>
+        <v>0.363276</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.511908</v>
+        <v>0.357336</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.499114</v>
+        <v>0.336668</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.177993</v>
+        <v>0.305292</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.174709</v>
       </c>
     </row>
     <row r="5">
@@ -1502,22 +1575,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.509284</v>
+        <v>0.34348</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.512656</v>
+        <v>0.351908</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.515756</v>
+        <v>0.360201</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.518181</v>
+        <v>0.367467</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.517415</v>
+        <v>0.368065</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.354522</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.174696</v>
       </c>
     </row>
     <row r="6">
@@ -1525,22 +1601,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.497442</v>
+        <v>0.317277</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.5034380000000001</v>
+        <v>0.329918</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.509286</v>
+        <v>0.343454</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.514854</v>
+        <v>0.357665</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.51884</v>
+        <v>0.369676</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.366559</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.174693</v>
       </c>
     </row>
     <row r="7">
@@ -1548,22 +1627,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.485185</v>
+        <v>0.294672</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.493792</v>
+        <v>0.310138</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.502116</v>
+        <v>0.327081</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.510412</v>
+        <v>0.346232</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.517763</v>
+        <v>0.365864</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.177988</v>
+        <v>0.370109</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.174689</v>
       </c>
     </row>
     <row r="8">
@@ -1571,22 +1653,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.472241</v>
+        <v>0.274579</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.483754</v>
+        <v>0.292322</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.494866</v>
+        <v>0.312242</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.505745</v>
+        <v>0.335182</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.515954</v>
+        <v>0.360639</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.370714</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.174695</v>
       </c>
     </row>
     <row r="9">
@@ -1594,22 +1679,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.459365</v>
+        <v>0.257385</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.473397</v>
+        <v>0.276269</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.487421</v>
+        <v>0.298588</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.50093</v>
+        <v>0.324582</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.513819</v>
+        <v>0.354907</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.369421</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.174692</v>
       </c>
     </row>
     <row r="10">
@@ -1617,22 +1705,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.446312</v>
+        <v>0.242063</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.463127</v>
+        <v>0.262194</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.479721</v>
+        <v>0.28587</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.495954</v>
+        <v>0.314433</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.511526</v>
+        <v>0.349044</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.367298</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.174691</v>
       </c>
     </row>
     <row r="11">
@@ -1640,22 +1731,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.433206</v>
+        <v>0.228299</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.452681</v>
+        <v>0.249336</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.472072</v>
+        <v>0.274394</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.491045</v>
+        <v>0.305111</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.509188</v>
+        <v>0.343325</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.177987</v>
+        <v>0.36477</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.174687</v>
       </c>
     </row>
   </sheetData>
@@ -1684,7 +1778,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -1718,22 +1812,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.375381</v>
+        <v>0.721296</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.375408</v>
+        <v>0.720206</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.374819</v>
+        <v>0.716857</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.372681</v>
+        <v>0.707013</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.364118</v>
+        <v>0.672125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.128306</v>
+        <v>0.182393</v>
       </c>
     </row>
     <row r="5">
@@ -1741,22 +1835,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.369639</v>
+        <v>0.716266</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.371995</v>
+        <v>0.721016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.374193</v>
+        <v>0.725425</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.376003</v>
+        <v>0.728177</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.375864</v>
+        <v>0.723059</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.128304</v>
+        <v>0.182389</v>
       </c>
     </row>
     <row r="6">
@@ -1764,22 +1858,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.361244</v>
+        <v>0.698484</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.365423</v>
+        <v>0.707616</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.369509</v>
+        <v>0.716408</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.373419</v>
+        <v>0.724815</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.376431</v>
+        <v>0.72904</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182388</v>
       </c>
     </row>
     <row r="7">
@@ -1787,22 +1881,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.352561</v>
+        <v>0.6793630000000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.358622</v>
+        <v>0.692587</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.364454</v>
+        <v>0.705593</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.370239</v>
+        <v>0.718198</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.375481</v>
+        <v>0.728581</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.182403</v>
       </c>
     </row>
     <row r="8">
@@ -1810,22 +1904,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.343355</v>
+        <v>0.660434</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.351511</v>
+        <v>0.677283</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.359337</v>
+        <v>0.694479</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.366944</v>
+        <v>0.7111769999999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.374115</v>
+        <v>0.726436</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182386</v>
       </c>
     </row>
     <row r="9">
@@ -1833,22 +1927,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.334158</v>
+        <v>0.64097</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.344156</v>
+        <v>0.662505</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.354078</v>
+        <v>0.6832780000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.363558</v>
+        <v>0.703989</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.372577</v>
+        <v>0.723368</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182387</v>
       </c>
     </row>
     <row r="10">
@@ -1856,22 +1950,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.324795</v>
+        <v>0.622152</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.336824</v>
+        <v>0.6469510000000001</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.348606</v>
+        <v>0.671573</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.360058</v>
+        <v>0.696204</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.370937</v>
+        <v>0.719983</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182385</v>
       </c>
     </row>
     <row r="11">
@@ -1879,22 +1973,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.315368</v>
+        <v>0.604131</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.329339</v>
+        <v>0.631347</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.343169</v>
+        <v>0.659758</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.356587</v>
+        <v>0.68865</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.369291</v>
+        <v>0.716566</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.182391</v>
       </c>
     </row>
   </sheetData>
@@ -1923,6 +2017,484 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.51635</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.516308</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.515298</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.511908</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.499114</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.177993</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.509284</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.512656</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.515756</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.518181</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.517415</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.17799</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.497442</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.5034380000000001</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.509286</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.514854</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.51884</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.17799</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.485185</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.493792</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.502116</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.510412</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.517763</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.177988</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.472241</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.483754</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.494866</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.505745</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.515954</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.177989</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.459365</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.473397</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.487421</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.50093</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.513819</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.177989</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.446312</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.463127</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.479721</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.495954</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.511526</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.177989</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.433206</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.452681</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.472072</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.491045</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.509188</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.177987</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.375381</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.375408</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.374819</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.372681</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.364118</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.128306</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.369639</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.371995</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.374193</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.376003</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.375864</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.128304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.361244</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.365423</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.369509</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.373419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.376431</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.352561</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.358622</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.364454</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.370239</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.375481</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.343355</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.351511</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.359337</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.366944</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.374115</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.334158</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.344156</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.354078</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.363558</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.372577</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.324795</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.336824</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.348606</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.360058</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.370937</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.315368</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.329339</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.343169</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.356587</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.369291</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
           <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add ITO 50 nm sweep results to raw-data spreadsheet
ITO thinned 150 -> 50 nm (ETL/HTL 500 nm, Ag):
- n=1.8:  EQE_sub 0.884 -> 0.890, best SL EQE 0.810 -> 0.830
- n=1.51: EQE_sub 0.565 -> 0.580, best SL EQE 0.533 -> 0.555
Thinner ITO recovers roughly half of the ITO absorption loss
identified by the k=0 diagnostic.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -10,12 +10,14 @@
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="n1.80_ETLHTL500" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="n1.51_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="n1.80_ETLHTL500_Al" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="n1.51_ETLHTL500_Al" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="n1.80_ETLHTL80" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="n1.51_ETLHTL80" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="n1.51_ETLHTL150" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="n1.51_ETLHTL200" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="n1.80_t500_ITO50" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="n1.51_t500_ITO50" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="n1.80_ETLHTL500_Al" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.51_ETLHTL500_Al" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="n1.80_ETLHTL80" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="n1.51_ETLHTL80" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="n1.51_ETLHTL150" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="n1.51_ETLHTL200" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,73 +618,587 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL80</t>
+          <t>n1.80_t500_ITO50</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.1854</v>
+        <v>0.205</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.8902</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL80</t>
+          <t>n1.51_t500_ITO50</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.222</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.5525</v>
+        <v>0.5802</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL150</t>
+          <t>n1.80_ETLHTL80</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.1311</v>
+        <v>0.1854</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.8097</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>n1.51_ETLHTL80</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>0.1865</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>0.5525</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>n1.51_ETLHTL150</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>0.1311</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0.4005</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>n1.51_ETLHTL200</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C18" s="2" t="n">
         <v>0.3347</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D18" s="2" t="n">
         <v>0.5671</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.375381</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.375408</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.374819</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.372681</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.364118</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.128306</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.369639</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.371995</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.374193</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.376003</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.375864</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.128304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.361244</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.365423</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.369509</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.373419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.376431</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.352561</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.358622</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.364454</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.370239</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.375481</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.343355</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.351511</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.359337</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.366944</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.374115</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.334158</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.344156</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.354078</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.363558</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.372577</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.324795</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.336824</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.348606</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.360058</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.370937</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.315368</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.329339</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.343169</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.356587</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.369291</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.536658</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.537242</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.537309</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.5361089999999999</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.529569</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.325075</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.5270319999999999</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.530506</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.53384</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.5369159999999999</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.538465</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.32507</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.515095</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.521091</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.526971</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.532743</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.537843</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.325069</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.502815</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.511445</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.519797</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.52811</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.535994</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.325067</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.489808</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.501407</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.512553</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.523421</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.533863</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.325069</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.476786</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.49101</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.5051330000000001</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.518642</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.531596</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.325068</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.46353</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.480659</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.497412</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.513698</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.529244</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.325068</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.450183</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.470059</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.489716</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.508785</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.526905</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.325065</v>
       </c>
     </row>
   </sheetData>
@@ -1245,7 +1761,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -1282,25 +1798,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.527973</v>
+        <v>0.824137</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.527058</v>
+        <v>0.823284</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.522398</v>
+        <v>0.820526</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.508132</v>
+        <v>0.811936</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.464831</v>
+        <v>0.778237</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.401885</v>
+        <v>0.70441</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.176671</v>
+        <v>0.207041</v>
       </c>
     </row>
     <row r="5">
@@ -1308,25 +1824,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.513765</v>
+        <v>0.818106</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.523353</v>
+        <v>0.82236</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.533013</v>
+        <v>0.826344</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.539902</v>
+        <v>0.829004</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.53354</v>
+        <v>0.825467</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5025810000000001</v>
+        <v>0.807518</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.176663</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="6">
@@ -1334,25 +1850,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.481836</v>
+        <v>0.801698</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.497634</v>
+        <v>0.810121</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.5140169999999999</v>
+        <v>0.818107</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.531281</v>
+        <v>0.82559</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.542503</v>
+        <v>0.829821</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.529126</v>
+        <v>0.823088</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.176665</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="7">
@@ -1360,25 +1876,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.452262</v>
+        <v>0.783354</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.472202</v>
+        <v>0.796052</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.494101</v>
+        <v>0.808265</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.517697</v>
+        <v>0.819679</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5401</v>
+        <v>0.829047</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.539558</v>
+        <v>0.828209</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.176684</v>
+        <v>0.207043</v>
       </c>
     </row>
     <row r="8">
@@ -1386,25 +1902,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.426585</v>
+        <v>0.764553</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.4493</v>
+        <v>0.7812829999999999</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.475345</v>
+        <v>0.797841</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.504194</v>
+        <v>0.813349</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.534932</v>
+        <v>0.8270110000000001</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.5428269999999999</v>
+        <v>0.829836</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.176655</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="9">
@@ -1412,25 +1928,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.402791</v>
+        <v>0.744617</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.429294</v>
+        <v>0.7665960000000001</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.458065</v>
+        <v>0.787125</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.491371</v>
+        <v>0.806735</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.528176</v>
+        <v>0.824228</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.5435759999999999</v>
+        <v>0.830226</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.176657</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="10">
@@ -1438,25 +1954,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.381897</v>
+        <v>0.724892</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.409937</v>
+        <v>0.750803</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.441454</v>
+        <v>0.775667</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.478134</v>
+        <v>0.799481</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.521226</v>
+        <v>0.82123</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.541695</v>
+        <v>0.829608</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.176651</v>
+        <v>0.207036</v>
       </c>
     </row>
     <row r="11">
@@ -1464,25 +1980,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.363437</v>
+        <v>0.705694</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.391913</v>
+        <v>0.73454</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.425692</v>
+        <v>0.763796</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.466244</v>
+        <v>0.7923</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.514435</v>
+        <v>0.818198</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.53949</v>
+        <v>0.828788</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.176667</v>
+        <v>0.20704</v>
       </c>
     </row>
   </sheetData>
@@ -1512,7 +2028,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -1549,25 +2065,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.364003</v>
+        <v>0.55288</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.364627</v>
+        <v>0.552984</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.363276</v>
+        <v>0.552415</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.357336</v>
+        <v>0.5501470000000001</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.336668</v>
+        <v>0.540554</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.305292</v>
+        <v>0.516624</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.174709</v>
+        <v>0.216258</v>
       </c>
     </row>
     <row r="5">
@@ -1575,25 +2091,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.34348</v>
+        <v>0.546467</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.351908</v>
+        <v>0.549218</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.360201</v>
+        <v>0.551769</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.367467</v>
+        <v>0.553877</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.368065</v>
+        <v>0.5538459999999999</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.354522</v>
+        <v>0.5488420000000001</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.174696</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="6">
@@ -1601,25 +2117,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.317277</v>
+        <v>0.5365799999999999</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.329918</v>
+        <v>0.541612</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.343454</v>
+        <v>0.546428</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.357665</v>
+        <v>0.550978</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.369676</v>
+        <v>0.554465</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.366559</v>
+        <v>0.553283</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.174693</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="7">
@@ -1627,25 +2143,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.294672</v>
+        <v>0.525908</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.310138</v>
+        <v>0.533448</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.327081</v>
+        <v>0.540516</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.346232</v>
+        <v>0.547341</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.365864</v>
+        <v>0.553399</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.370109</v>
+        <v>0.55449</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.174689</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="8">
@@ -1653,25 +2169,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.274579</v>
+        <v>0.514146</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.292322</v>
+        <v>0.524638</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.312242</v>
+        <v>0.534377</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.335182</v>
+        <v>0.543524</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.360639</v>
+        <v>0.551862</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.370714</v>
+        <v>0.554735</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.174695</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="9">
@@ -1679,25 +2195,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.257385</v>
+        <v>0.502013</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.276269</v>
+        <v>0.515224</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.298588</v>
+        <v>0.527905</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.324582</v>
+        <v>0.539524</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.354907</v>
+        <v>0.550112</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.369421</v>
+        <v>0.554397</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.174692</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="10">
@@ -1705,25 +2221,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.242063</v>
+        <v>0.489356</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.262194</v>
+        <v>0.505612</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.28587</v>
+        <v>0.52102</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.314433</v>
+        <v>0.535322</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.349044</v>
+        <v>0.548245</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.367298</v>
+        <v>0.553799</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.174691</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="11">
@@ -1731,25 +2247,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.228299</v>
+        <v>0.476366</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.249336</v>
+        <v>0.495584</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.274394</v>
+        <v>0.514006</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.305111</v>
+        <v>0.531089</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.343325</v>
+        <v>0.5463479999999999</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.36477</v>
+        <v>0.553071</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.174687</v>
+        <v>0.216253</v>
       </c>
     </row>
   </sheetData>
@@ -1763,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1773,12 +2289,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -1804,6 +2321,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1812,22 +2332,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.721296</v>
+        <v>0.527973</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.720206</v>
+        <v>0.527058</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.716857</v>
+        <v>0.522398</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.707013</v>
+        <v>0.508132</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.672125</v>
+        <v>0.464831</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.182393</v>
+        <v>0.401885</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.176671</v>
       </c>
     </row>
     <row r="5">
@@ -1835,22 +2358,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.716266</v>
+        <v>0.513765</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.721016</v>
+        <v>0.523353</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.725425</v>
+        <v>0.533013</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.728177</v>
+        <v>0.539902</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.723059</v>
+        <v>0.53354</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.182389</v>
+        <v>0.5025810000000001</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.176663</v>
       </c>
     </row>
     <row r="6">
@@ -1858,22 +2384,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.698484</v>
+        <v>0.481836</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.707616</v>
+        <v>0.497634</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.716408</v>
+        <v>0.5140169999999999</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.724815</v>
+        <v>0.531281</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.72904</v>
+        <v>0.542503</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.182388</v>
+        <v>0.529126</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.176665</v>
       </c>
     </row>
     <row r="7">
@@ -1881,22 +2410,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6793630000000001</v>
+        <v>0.452262</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.692587</v>
+        <v>0.472202</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.705593</v>
+        <v>0.494101</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.718198</v>
+        <v>0.517697</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.728581</v>
+        <v>0.5401</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.182403</v>
+        <v>0.539558</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.176684</v>
       </c>
     </row>
     <row r="8">
@@ -1904,22 +2436,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.660434</v>
+        <v>0.426585</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.677283</v>
+        <v>0.4493</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.694479</v>
+        <v>0.475345</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.7111769999999999</v>
+        <v>0.504194</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.726436</v>
+        <v>0.534932</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.182386</v>
+        <v>0.5428269999999999</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.176655</v>
       </c>
     </row>
     <row r="9">
@@ -1927,22 +2462,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.64097</v>
+        <v>0.402791</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.662505</v>
+        <v>0.429294</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.6832780000000001</v>
+        <v>0.458065</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.703989</v>
+        <v>0.491371</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.723368</v>
+        <v>0.528176</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.182387</v>
+        <v>0.5435759999999999</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.176657</v>
       </c>
     </row>
     <row r="10">
@@ -1950,22 +2488,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.622152</v>
+        <v>0.381897</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6469510000000001</v>
+        <v>0.409937</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671573</v>
+        <v>0.441454</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.696204</v>
+        <v>0.478134</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.719983</v>
+        <v>0.521226</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.182385</v>
+        <v>0.541695</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.176651</v>
       </c>
     </row>
     <row r="11">
@@ -1973,22 +2514,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.604131</v>
+        <v>0.363437</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.631347</v>
+        <v>0.391913</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.659758</v>
+        <v>0.425692</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.68865</v>
+        <v>0.466244</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.716566</v>
+        <v>0.514435</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.182391</v>
+        <v>0.53949</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.176667</v>
       </c>
     </row>
   </sheetData>
@@ -2002,7 +2546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2012,12 +2556,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -2043,6 +2588,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2051,22 +2599,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.51635</v>
+        <v>0.364003</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.516308</v>
+        <v>0.364627</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.515298</v>
+        <v>0.363276</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.511908</v>
+        <v>0.357336</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.499114</v>
+        <v>0.336668</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.177993</v>
+        <v>0.305292</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.174709</v>
       </c>
     </row>
     <row r="5">
@@ -2074,22 +2625,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.509284</v>
+        <v>0.34348</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.512656</v>
+        <v>0.351908</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.515756</v>
+        <v>0.360201</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.518181</v>
+        <v>0.367467</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.517415</v>
+        <v>0.368065</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.354522</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.174696</v>
       </c>
     </row>
     <row r="6">
@@ -2097,22 +2651,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.497442</v>
+        <v>0.317277</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.5034380000000001</v>
+        <v>0.329918</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.509286</v>
+        <v>0.343454</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.514854</v>
+        <v>0.357665</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.51884</v>
+        <v>0.369676</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.366559</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.174693</v>
       </c>
     </row>
     <row r="7">
@@ -2120,22 +2677,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.485185</v>
+        <v>0.294672</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.493792</v>
+        <v>0.310138</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.502116</v>
+        <v>0.327081</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.510412</v>
+        <v>0.346232</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.517763</v>
+        <v>0.365864</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.177988</v>
+        <v>0.370109</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.174689</v>
       </c>
     </row>
     <row r="8">
@@ -2143,22 +2703,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.472241</v>
+        <v>0.274579</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.483754</v>
+        <v>0.292322</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.494866</v>
+        <v>0.312242</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.505745</v>
+        <v>0.335182</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.515954</v>
+        <v>0.360639</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.370714</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.174695</v>
       </c>
     </row>
     <row r="9">
@@ -2166,22 +2729,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.459365</v>
+        <v>0.257385</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.473397</v>
+        <v>0.276269</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.487421</v>
+        <v>0.298588</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.50093</v>
+        <v>0.324582</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.513819</v>
+        <v>0.354907</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.369421</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.174692</v>
       </c>
     </row>
     <row r="10">
@@ -2189,22 +2755,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.446312</v>
+        <v>0.242063</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.463127</v>
+        <v>0.262194</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.479721</v>
+        <v>0.28587</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.495954</v>
+        <v>0.314433</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.511526</v>
+        <v>0.349044</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.367298</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.174691</v>
       </c>
     </row>
     <row r="11">
@@ -2212,22 +2781,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.433206</v>
+        <v>0.228299</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.452681</v>
+        <v>0.249336</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.472072</v>
+        <v>0.274394</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.491045</v>
+        <v>0.305111</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.509188</v>
+        <v>0.343325</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.177987</v>
+        <v>0.36477</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.174687</v>
       </c>
     </row>
   </sheetData>
@@ -2256,7 +2828,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -2290,22 +2862,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.375381</v>
+        <v>0.721296</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.375408</v>
+        <v>0.720206</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.374819</v>
+        <v>0.716857</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.372681</v>
+        <v>0.707013</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.364118</v>
+        <v>0.672125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.128306</v>
+        <v>0.182393</v>
       </c>
     </row>
     <row r="5">
@@ -2313,22 +2885,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.369639</v>
+        <v>0.716266</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.371995</v>
+        <v>0.721016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.374193</v>
+        <v>0.725425</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.376003</v>
+        <v>0.728177</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.375864</v>
+        <v>0.723059</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.128304</v>
+        <v>0.182389</v>
       </c>
     </row>
     <row r="6">
@@ -2336,22 +2908,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.361244</v>
+        <v>0.698484</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.365423</v>
+        <v>0.707616</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.369509</v>
+        <v>0.716408</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.373419</v>
+        <v>0.724815</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.376431</v>
+        <v>0.72904</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182388</v>
       </c>
     </row>
     <row r="7">
@@ -2359,22 +2931,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.352561</v>
+        <v>0.6793630000000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.358622</v>
+        <v>0.692587</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.364454</v>
+        <v>0.705593</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.370239</v>
+        <v>0.718198</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.375481</v>
+        <v>0.728581</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.182403</v>
       </c>
     </row>
     <row r="8">
@@ -2382,22 +2954,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.343355</v>
+        <v>0.660434</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.351511</v>
+        <v>0.677283</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.359337</v>
+        <v>0.694479</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.366944</v>
+        <v>0.7111769999999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.374115</v>
+        <v>0.726436</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182386</v>
       </c>
     </row>
     <row r="9">
@@ -2405,22 +2977,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.334158</v>
+        <v>0.64097</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.344156</v>
+        <v>0.662505</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.354078</v>
+        <v>0.6832780000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.363558</v>
+        <v>0.703989</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.372577</v>
+        <v>0.723368</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182387</v>
       </c>
     </row>
     <row r="10">
@@ -2428,22 +3000,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.324795</v>
+        <v>0.622152</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.336824</v>
+        <v>0.6469510000000001</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.348606</v>
+        <v>0.671573</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.360058</v>
+        <v>0.696204</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.370937</v>
+        <v>0.719983</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.182385</v>
       </c>
     </row>
     <row r="11">
@@ -2451,22 +3023,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.315368</v>
+        <v>0.604131</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.329339</v>
+        <v>0.631347</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.343169</v>
+        <v>0.659758</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.356587</v>
+        <v>0.68865</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.369291</v>
+        <v>0.716566</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.182391</v>
       </c>
     </row>
   </sheetData>
@@ -2495,7 +3067,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -2529,22 +3101,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.536658</v>
+        <v>0.51635</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.537242</v>
+        <v>0.516308</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.537309</v>
+        <v>0.515298</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.5361089999999999</v>
+        <v>0.511908</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.529569</v>
+        <v>0.499114</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.325075</v>
+        <v>0.177993</v>
       </c>
     </row>
     <row r="5">
@@ -2552,22 +3124,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.5270319999999999</v>
+        <v>0.509284</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.530506</v>
+        <v>0.512656</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.53384</v>
+        <v>0.515756</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.5369159999999999</v>
+        <v>0.518181</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.538465</v>
+        <v>0.517415</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.32507</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="6">
@@ -2575,22 +3147,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.515095</v>
+        <v>0.497442</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.521091</v>
+        <v>0.5034380000000001</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.526971</v>
+        <v>0.509286</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.532743</v>
+        <v>0.514854</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.537843</v>
+        <v>0.51884</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.325069</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="7">
@@ -2598,22 +3170,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.502815</v>
+        <v>0.485185</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.511445</v>
+        <v>0.493792</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.519797</v>
+        <v>0.502116</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.52811</v>
+        <v>0.510412</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.535994</v>
+        <v>0.517763</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.325067</v>
+        <v>0.177988</v>
       </c>
     </row>
     <row r="8">
@@ -2621,22 +3193,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.489808</v>
+        <v>0.472241</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.501407</v>
+        <v>0.483754</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.512553</v>
+        <v>0.494866</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.523421</v>
+        <v>0.505745</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.533863</v>
+        <v>0.515954</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.325069</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="9">
@@ -2644,22 +3216,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.476786</v>
+        <v>0.459365</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.49101</v>
+        <v>0.473397</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.5051330000000001</v>
+        <v>0.487421</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.518642</v>
+        <v>0.50093</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.531596</v>
+        <v>0.513819</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.325068</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="10">
@@ -2667,22 +3239,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.46353</v>
+        <v>0.446312</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.480659</v>
+        <v>0.463127</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.497412</v>
+        <v>0.479721</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.513698</v>
+        <v>0.495954</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.529244</v>
+        <v>0.511526</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.325068</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="11">
@@ -2690,22 +3262,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.450183</v>
+        <v>0.433206</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.470059</v>
+        <v>0.452681</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.489716</v>
+        <v>0.472072</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.508785</v>
+        <v>0.491045</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.526905</v>
+        <v>0.509188</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.325065</v>
+        <v>0.177987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ideal all-n=1.8 sweep results to raw-data spreadsheet
Fully index-matched organics (n=1.8 lossless): EQE_sub = 0.966,
scattering layer reaches 0.895 (x5.0 vs planar 0.178).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="n1.80_ETLHTL500" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="n1.51_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="n1.80_t500_ITO50" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="n1.51_t500_ITO50" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="n1.80_ETLHTL500_Al" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="n1.51_ETLHTL500_Al" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="n1.80_ETLHTL80" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="n1.51_ETLHTL80" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="n1.51_ETLHTL150" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="n1.51_ETLHTL200" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ideal_n1.8_ITO50" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="n1.80_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="n1.51_ETLHTL500" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="n1.80_t500_ITO50" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="n1.51_t500_ITO50" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.80_ETLHTL500_Al" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="n1.51_ETLHTL500_Al" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="n1.80_ETLHTL80" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="n1.51_ETLHTL80" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="n1.51_ETLHTL150" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="n1.51_ETLHTL200" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -546,180 +547,198 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL500</t>
+          <t>ideal_n1.8_ITO50</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>IDEAL: all organics n=1.8 lossless, n_sub=n_SL=1.80, ETL/HTL 500 nm, Ag, ITO 50 nm</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.2036</v>
+        <v>0.1778</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.8845</v>
+        <v>0.9665</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL500</t>
+          <t>n1.80_ETLHTL500</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.2126</v>
+        <v>0.2036</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.5649</v>
+        <v>0.8845</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL500_Al</t>
+          <t>n1.51_ETLHTL500</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.1778</v>
+        <v>0.2126</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.7775</v>
+        <v>0.5649</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL500_Al</t>
+          <t>n1.80_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.1794</v>
+        <v>0.1778</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.4801</v>
+        <v>0.7775</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>n1.80_t500_ITO50</t>
+          <t>n1.51_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.205</v>
+        <v>0.1794</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.8902</v>
+        <v>0.4801</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>n1.51_t500_ITO50</t>
+          <t>n1.80_t500_ITO50</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.222</v>
+        <v>0.205</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.5802</v>
+        <v>0.8902</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL80</t>
+          <t>n1.51_t500_ITO50</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.1854</v>
+        <v>0.222</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.5802</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL80</t>
+          <t>n1.80_ETLHTL80</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.1854</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.5525</v>
+        <v>0.8097</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL150</t>
+          <t>n1.51_ETLHTL80</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.1311</v>
+        <v>0.1865</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.5525</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>n1.51_ETLHTL150</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>0.1311</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>0.4005</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>n1.51_ETLHTL200</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C19" s="2" t="n">
         <v>0.3347</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D19" s="2" t="n">
         <v>0.5671</v>
       </c>
     </row>
@@ -749,7 +768,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -783,22 +802,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.375381</v>
+        <v>0.51635</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.375408</v>
+        <v>0.516308</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.374819</v>
+        <v>0.515298</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.372681</v>
+        <v>0.511908</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.364118</v>
+        <v>0.499114</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.128306</v>
+        <v>0.177993</v>
       </c>
     </row>
     <row r="5">
@@ -806,22 +825,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.369639</v>
+        <v>0.509284</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.371995</v>
+        <v>0.512656</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.374193</v>
+        <v>0.515756</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.376003</v>
+        <v>0.518181</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.375864</v>
+        <v>0.517415</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.128304</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="6">
@@ -829,22 +848,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.361244</v>
+        <v>0.497442</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.365423</v>
+        <v>0.5034380000000001</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.369509</v>
+        <v>0.509286</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.373419</v>
+        <v>0.514854</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.376431</v>
+        <v>0.51884</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="7">
@@ -852,22 +871,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.352561</v>
+        <v>0.485185</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.358622</v>
+        <v>0.493792</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.364454</v>
+        <v>0.502116</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.370239</v>
+        <v>0.510412</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.375481</v>
+        <v>0.517763</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177988</v>
       </c>
     </row>
     <row r="8">
@@ -875,22 +894,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.343355</v>
+        <v>0.472241</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.351511</v>
+        <v>0.483754</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.359337</v>
+        <v>0.494866</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.366944</v>
+        <v>0.505745</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.374115</v>
+        <v>0.515954</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="9">
@@ -898,22 +917,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.334158</v>
+        <v>0.459365</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.344156</v>
+        <v>0.473397</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.354078</v>
+        <v>0.487421</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.363558</v>
+        <v>0.50093</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.372577</v>
+        <v>0.513819</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="10">
@@ -921,22 +940,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.324795</v>
+        <v>0.446312</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.336824</v>
+        <v>0.463127</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.348606</v>
+        <v>0.479721</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.360058</v>
+        <v>0.495954</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.370937</v>
+        <v>0.511526</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="11">
@@ -944,22 +963,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.315368</v>
+        <v>0.433206</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.329339</v>
+        <v>0.452681</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.343169</v>
+        <v>0.472072</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.356587</v>
+        <v>0.491045</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.369291</v>
+        <v>0.509188</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177987</v>
       </c>
     </row>
   </sheetData>
@@ -988,6 +1007,245 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.375381</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.375408</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.374819</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.372681</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.364118</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.128306</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.369639</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.371995</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.374193</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.376003</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.375864</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.128304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.361244</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.365423</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.369509</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.373419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.376431</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.352561</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.358622</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.364454</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.370239</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.375481</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.343355</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.351511</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.359337</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.366944</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.374115</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.334158</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.344156</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.354078</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.363558</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.372577</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.324795</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.336824</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.348606</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.360058</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.370937</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.315368</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.329339</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.343169</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.356587</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.369291</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
           <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
@@ -1222,12 +1480,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>EQE (absolute), IDEAL: all organics n=1.8 lossless, n_sub=n_SL=1.80, ETL/HTL 500 nm, Ag, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -1264,25 +1523,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.802346</v>
+        <v>0.889194</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.8015099999999999</v>
+        <v>0.887853</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.798539</v>
+        <v>0.884225</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.789211</v>
+        <v>0.873607</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.753881</v>
+        <v>0.833449</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.679825</v>
+        <v>0.747165</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.206945</v>
+        <v>0.18014</v>
       </c>
     </row>
     <row r="5">
@@ -1290,25 +1549,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.795335</v>
+        <v>0.883114</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.800245</v>
+        <v>0.8877</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.804915</v>
+        <v>0.891823</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.808075</v>
+        <v>0.894359</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.804253</v>
+        <v>0.889249</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.784639</v>
+        <v>0.8673959999999999</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.206942</v>
+        <v>0.180139</v>
       </c>
     </row>
     <row r="6">
@@ -1316,25 +1575,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.77694</v>
+        <v>0.8650640000000001</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.786347</v>
+        <v>0.874265</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.795369</v>
+        <v>0.882879</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.804036</v>
+        <v>0.8908700000000001</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.809096</v>
+        <v>0.894853</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.80163</v>
+        <v>0.8860980000000001</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.206943</v>
+        <v>0.180139</v>
       </c>
     </row>
     <row r="7">
@@ -1342,25 +1601,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.756964</v>
+        <v>0.844938</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.770733</v>
+        <v>0.858728</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.784267</v>
+        <v>0.87208</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.797227</v>
+        <v>0.884413</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.808132</v>
+        <v>0.894333</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.807364</v>
+        <v>0.892436</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.206948</v>
+        <v>0.180142</v>
       </c>
     </row>
     <row r="8">
@@ -1368,25 +1627,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.736989</v>
+        <v>0.8243509999999999</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.754758</v>
+        <v>0.842565</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.7727349999999999</v>
+        <v>0.860604</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.790002</v>
+        <v>0.877497</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.805727</v>
+        <v>0.892217</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.809157</v>
+        <v>0.894618</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.20694</v>
+        <v>0.180138</v>
       </c>
     </row>
     <row r="9">
@@ -1394,25 +1653,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.716166</v>
+        <v>0.802538</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.739159</v>
+        <v>0.826417</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.761058</v>
+        <v>0.848799</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.782603</v>
+        <v>0.8701680000000001</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.80248</v>
+        <v>0.889272</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.809593</v>
+        <v>0.895305</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.20694</v>
+        <v>0.180138</v>
       </c>
     </row>
     <row r="10">
@@ -1420,25 +1679,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.695902</v>
+        <v>0.781033</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.7226089999999999</v>
+        <v>0.809132</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.7487819999999999</v>
+        <v>0.836195</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.774516</v>
+        <v>0.862193</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.798996</v>
+        <v>0.885927</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.808812</v>
+        <v>0.894768</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.206939</v>
+        <v>0.180137</v>
       </c>
     </row>
     <row r="11">
@@ -1446,25 +1705,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.676357</v>
+        <v>0.760117</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.705797</v>
+        <v>0.791423</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.736194</v>
+        <v>0.823246</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.766665</v>
+        <v>0.854282</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.7955179999999999</v>
+        <v>0.882641</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.807827</v>
+        <v>0.894007</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.206943</v>
+        <v>0.180139</v>
       </c>
     </row>
   </sheetData>
@@ -1488,13 +1747,12 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
     </row>
@@ -1531,25 +1789,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.530174</v>
+        <v>0.802346</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.530294</v>
+        <v>0.8015099999999999</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.529574</v>
+        <v>0.798539</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.526768</v>
+        <v>0.789211</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.515456</v>
+        <v>0.753881</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.489715</v>
+        <v>0.679825</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.206753</v>
+        <v>0.206945</v>
       </c>
     </row>
     <row r="5">
@@ -1557,25 +1815,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.522313</v>
+        <v>0.795335</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.525689</v>
+        <v>0.800245</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.528843</v>
+        <v>0.804915</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.531454</v>
+        <v>0.808075</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.531369</v>
+        <v>0.804253</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5251749999999999</v>
+        <v>0.784639</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.206942</v>
       </c>
     </row>
     <row r="6">
@@ -1583,25 +1841,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.510482</v>
+        <v>0.77694</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.516444</v>
+        <v>0.786347</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.522269</v>
+        <v>0.795369</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.527867</v>
+        <v>0.804036</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.532183</v>
+        <v>0.809096</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.530655</v>
+        <v>0.80163</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.206943</v>
       </c>
     </row>
     <row r="7">
@@ -1609,25 +1867,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.498234</v>
+        <v>0.756964</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.506833</v>
+        <v>0.770733</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.515134</v>
+        <v>0.784267</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.523386</v>
+        <v>0.797227</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.530869</v>
+        <v>0.808132</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.532184</v>
+        <v>0.807364</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.206948</v>
       </c>
     </row>
     <row r="8">
@@ -1635,25 +1893,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.485254</v>
+        <v>0.736989</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.496809</v>
+        <v>0.754758</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.507911</v>
+        <v>0.7727349999999999</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.51874</v>
+        <v>0.790002</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.528961</v>
+        <v>0.805727</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.532516</v>
+        <v>0.809157</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.20694</v>
       </c>
     </row>
     <row r="9">
@@ -1661,25 +1919,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.472283</v>
+        <v>0.716166</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.486424</v>
+        <v>0.739159</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.500487</v>
+        <v>0.761058</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.513952</v>
+        <v>0.782603</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.526794</v>
+        <v>0.80248</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.5321050000000001</v>
+        <v>0.809593</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.20694</v>
       </c>
     </row>
     <row r="10">
@@ -1687,25 +1945,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.459081</v>
+        <v>0.695902</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.476091</v>
+        <v>0.7226089999999999</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.492779</v>
+        <v>0.7487819999999999</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.509009</v>
+        <v>0.774516</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.524493</v>
+        <v>0.798996</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.531368</v>
+        <v>0.808812</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.206939</v>
       </c>
     </row>
     <row r="11">
@@ -1713,25 +1971,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.445793</v>
+        <v>0.676357</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.465539</v>
+        <v>0.705797</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.4851</v>
+        <v>0.736194</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.504113</v>
+        <v>0.766665</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.522168</v>
+        <v>0.7955179999999999</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.53046</v>
+        <v>0.807827</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.206747</v>
+        <v>0.206943</v>
       </c>
     </row>
   </sheetData>
@@ -1761,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
     </row>
@@ -1798,25 +2056,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.824137</v>
+        <v>0.530174</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.823284</v>
+        <v>0.530294</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.820526</v>
+        <v>0.529574</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.811936</v>
+        <v>0.526768</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.778237</v>
+        <v>0.515456</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.70441</v>
+        <v>0.489715</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.207041</v>
+        <v>0.206753</v>
       </c>
     </row>
     <row r="5">
@@ -1824,25 +2082,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.818106</v>
+        <v>0.522313</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.82236</v>
+        <v>0.525689</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.826344</v>
+        <v>0.528843</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.829004</v>
+        <v>0.531454</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825467</v>
+        <v>0.531369</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.807518</v>
+        <v>0.5251749999999999</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.207039</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="6">
@@ -1850,25 +2108,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.801698</v>
+        <v>0.510482</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.810121</v>
+        <v>0.516444</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.818107</v>
+        <v>0.522269</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.82559</v>
+        <v>0.527867</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.829821</v>
+        <v>0.532183</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.823088</v>
+        <v>0.530655</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.207039</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="7">
@@ -1876,25 +2134,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.783354</v>
+        <v>0.498234</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.796052</v>
+        <v>0.506833</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.808265</v>
+        <v>0.515134</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.819679</v>
+        <v>0.523386</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.829047</v>
+        <v>0.530869</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.828209</v>
+        <v>0.532184</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.207043</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="8">
@@ -1902,25 +2160,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.764553</v>
+        <v>0.485254</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.7812829999999999</v>
+        <v>0.496809</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.797841</v>
+        <v>0.507911</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.813349</v>
+        <v>0.51874</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.8270110000000001</v>
+        <v>0.528961</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.829836</v>
+        <v>0.532516</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.207037</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="9">
@@ -1928,25 +2186,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.744617</v>
+        <v>0.472283</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.7665960000000001</v>
+        <v>0.486424</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.787125</v>
+        <v>0.500487</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.806735</v>
+        <v>0.513952</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.824228</v>
+        <v>0.526794</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.830226</v>
+        <v>0.5321050000000001</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.207037</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="10">
@@ -1954,25 +2212,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.724892</v>
+        <v>0.459081</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.750803</v>
+        <v>0.476091</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.775667</v>
+        <v>0.492779</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.799481</v>
+        <v>0.509009</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.82123</v>
+        <v>0.524493</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.829608</v>
+        <v>0.531368</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.207036</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="11">
@@ -1980,25 +2238,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.705694</v>
+        <v>0.445793</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.73454</v>
+        <v>0.465539</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.763796</v>
+        <v>0.4851</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.7923</v>
+        <v>0.504113</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.818198</v>
+        <v>0.522168</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.828788</v>
+        <v>0.53046</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.20704</v>
+        <v>0.206747</v>
       </c>
     </row>
   </sheetData>
@@ -2028,7 +2286,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -2065,25 +2323,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.55288</v>
+        <v>0.824137</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.552984</v>
+        <v>0.823284</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.552415</v>
+        <v>0.820526</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.5501470000000001</v>
+        <v>0.811936</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.540554</v>
+        <v>0.778237</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.516624</v>
+        <v>0.70441</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.216258</v>
+        <v>0.207041</v>
       </c>
     </row>
     <row r="5">
@@ -2091,25 +2349,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.546467</v>
+        <v>0.818106</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.549218</v>
+        <v>0.82236</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.551769</v>
+        <v>0.826344</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.553877</v>
+        <v>0.829004</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.5538459999999999</v>
+        <v>0.825467</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5488420000000001</v>
+        <v>0.807518</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="6">
@@ -2117,25 +2375,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.5365799999999999</v>
+        <v>0.801698</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.541612</v>
+        <v>0.810121</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.546428</v>
+        <v>0.818107</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.550978</v>
+        <v>0.82559</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.554465</v>
+        <v>0.829821</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.553283</v>
+        <v>0.823088</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="7">
@@ -2143,25 +2401,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.525908</v>
+        <v>0.783354</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.533448</v>
+        <v>0.796052</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.540516</v>
+        <v>0.808265</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.547341</v>
+        <v>0.819679</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.553399</v>
+        <v>0.829047</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.55449</v>
+        <v>0.828209</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207043</v>
       </c>
     </row>
     <row r="8">
@@ -2169,25 +2427,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.514146</v>
+        <v>0.764553</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.524638</v>
+        <v>0.7812829999999999</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.534377</v>
+        <v>0.797841</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.543524</v>
+        <v>0.813349</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.551862</v>
+        <v>0.8270110000000001</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.554735</v>
+        <v>0.829836</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="9">
@@ -2195,25 +2453,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.502013</v>
+        <v>0.744617</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.515224</v>
+        <v>0.7665960000000001</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.527905</v>
+        <v>0.787125</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.539524</v>
+        <v>0.806735</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.550112</v>
+        <v>0.824228</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.554397</v>
+        <v>0.830226</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="10">
@@ -2221,25 +2479,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.489356</v>
+        <v>0.724892</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.505612</v>
+        <v>0.750803</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.52102</v>
+        <v>0.775667</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.535322</v>
+        <v>0.799481</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.548245</v>
+        <v>0.82123</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.553799</v>
+        <v>0.829608</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207036</v>
       </c>
     </row>
     <row r="11">
@@ -2247,25 +2505,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.476366</v>
+        <v>0.705694</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.495584</v>
+        <v>0.73454</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.514006</v>
+        <v>0.763796</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.531089</v>
+        <v>0.7923</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.5463479999999999</v>
+        <v>0.818198</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.553071</v>
+        <v>0.828788</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.216253</v>
+        <v>0.20704</v>
       </c>
     </row>
   </sheetData>
@@ -2295,7 +2553,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -2332,25 +2590,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.527973</v>
+        <v>0.55288</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.527058</v>
+        <v>0.552984</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.522398</v>
+        <v>0.552415</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.508132</v>
+        <v>0.5501470000000001</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.464831</v>
+        <v>0.540554</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.401885</v>
+        <v>0.516624</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.176671</v>
+        <v>0.216258</v>
       </c>
     </row>
     <row r="5">
@@ -2358,25 +2616,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.513765</v>
+        <v>0.546467</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.523353</v>
+        <v>0.549218</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.533013</v>
+        <v>0.551769</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.539902</v>
+        <v>0.553877</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.53354</v>
+        <v>0.5538459999999999</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5025810000000001</v>
+        <v>0.5488420000000001</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.176663</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="6">
@@ -2384,25 +2642,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.481836</v>
+        <v>0.5365799999999999</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.497634</v>
+        <v>0.541612</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.5140169999999999</v>
+        <v>0.546428</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.531281</v>
+        <v>0.550978</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.542503</v>
+        <v>0.554465</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.529126</v>
+        <v>0.553283</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.176665</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="7">
@@ -2410,25 +2668,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.452262</v>
+        <v>0.525908</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.472202</v>
+        <v>0.533448</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.494101</v>
+        <v>0.540516</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.517697</v>
+        <v>0.547341</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5401</v>
+        <v>0.553399</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.539558</v>
+        <v>0.55449</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.176684</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="8">
@@ -2436,25 +2694,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.426585</v>
+        <v>0.514146</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.4493</v>
+        <v>0.524638</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.475345</v>
+        <v>0.534377</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.504194</v>
+        <v>0.543524</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.534932</v>
+        <v>0.551862</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.5428269999999999</v>
+        <v>0.554735</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.176655</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="9">
@@ -2462,25 +2720,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.402791</v>
+        <v>0.502013</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.429294</v>
+        <v>0.515224</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.458065</v>
+        <v>0.527905</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.491371</v>
+        <v>0.539524</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.528176</v>
+        <v>0.550112</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.5435759999999999</v>
+        <v>0.554397</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.176657</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="10">
@@ -2488,25 +2746,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.381897</v>
+        <v>0.489356</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.409937</v>
+        <v>0.505612</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.441454</v>
+        <v>0.52102</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.478134</v>
+        <v>0.535322</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.521226</v>
+        <v>0.548245</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.541695</v>
+        <v>0.553799</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.176651</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="11">
@@ -2514,25 +2772,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.363437</v>
+        <v>0.476366</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.391913</v>
+        <v>0.495584</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.425692</v>
+        <v>0.514006</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.466244</v>
+        <v>0.531089</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.514435</v>
+        <v>0.5463479999999999</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.53949</v>
+        <v>0.553071</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.176667</v>
+        <v>0.216253</v>
       </c>
     </row>
   </sheetData>
@@ -2562,7 +2820,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -2599,25 +2857,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.364003</v>
+        <v>0.527973</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.364627</v>
+        <v>0.527058</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.363276</v>
+        <v>0.522398</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.357336</v>
+        <v>0.508132</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.336668</v>
+        <v>0.464831</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.305292</v>
+        <v>0.401885</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.174709</v>
+        <v>0.176671</v>
       </c>
     </row>
     <row r="5">
@@ -2625,25 +2883,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.34348</v>
+        <v>0.513765</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.351908</v>
+        <v>0.523353</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.360201</v>
+        <v>0.533013</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.367467</v>
+        <v>0.539902</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.368065</v>
+        <v>0.53354</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.354522</v>
+        <v>0.5025810000000001</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.174696</v>
+        <v>0.176663</v>
       </c>
     </row>
     <row r="6">
@@ -2651,25 +2909,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.317277</v>
+        <v>0.481836</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.329918</v>
+        <v>0.497634</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.343454</v>
+        <v>0.5140169999999999</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.357665</v>
+        <v>0.531281</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.369676</v>
+        <v>0.542503</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.366559</v>
+        <v>0.529126</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.174693</v>
+        <v>0.176665</v>
       </c>
     </row>
     <row r="7">
@@ -2677,25 +2935,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.294672</v>
+        <v>0.452262</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.310138</v>
+        <v>0.472202</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.327081</v>
+        <v>0.494101</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.346232</v>
+        <v>0.517697</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.365864</v>
+        <v>0.5401</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.370109</v>
+        <v>0.539558</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.174689</v>
+        <v>0.176684</v>
       </c>
     </row>
     <row r="8">
@@ -2703,25 +2961,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.274579</v>
+        <v>0.426585</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.292322</v>
+        <v>0.4493</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.312242</v>
+        <v>0.475345</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.335182</v>
+        <v>0.504194</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.360639</v>
+        <v>0.534932</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.370714</v>
+        <v>0.5428269999999999</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.174695</v>
+        <v>0.176655</v>
       </c>
     </row>
     <row r="9">
@@ -2729,25 +2987,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.257385</v>
+        <v>0.402791</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.276269</v>
+        <v>0.429294</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.298588</v>
+        <v>0.458065</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.324582</v>
+        <v>0.491371</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.354907</v>
+        <v>0.528176</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.369421</v>
+        <v>0.5435759999999999</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.174692</v>
+        <v>0.176657</v>
       </c>
     </row>
     <row r="10">
@@ -2755,25 +3013,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.242063</v>
+        <v>0.381897</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.262194</v>
+        <v>0.409937</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.28587</v>
+        <v>0.441454</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.314433</v>
+        <v>0.478134</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.349044</v>
+        <v>0.521226</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.367298</v>
+        <v>0.541695</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.174691</v>
+        <v>0.176651</v>
       </c>
     </row>
     <row r="11">
@@ -2781,25 +3039,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.228299</v>
+        <v>0.363437</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.249336</v>
+        <v>0.391913</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.274394</v>
+        <v>0.425692</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.305111</v>
+        <v>0.466244</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.343325</v>
+        <v>0.514435</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.36477</v>
+        <v>0.53949</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.174687</v>
+        <v>0.176667</v>
       </c>
     </row>
   </sheetData>
@@ -2813,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2823,12 +3081,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -2854,6 +3113,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2862,22 +3124,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.721296</v>
+        <v>0.364003</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.720206</v>
+        <v>0.364627</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.716857</v>
+        <v>0.363276</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.707013</v>
+        <v>0.357336</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.672125</v>
+        <v>0.336668</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.182393</v>
+        <v>0.305292</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.174709</v>
       </c>
     </row>
     <row r="5">
@@ -2885,22 +3150,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.716266</v>
+        <v>0.34348</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.721016</v>
+        <v>0.351908</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.725425</v>
+        <v>0.360201</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.728177</v>
+        <v>0.367467</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.723059</v>
+        <v>0.368065</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.182389</v>
+        <v>0.354522</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.174696</v>
       </c>
     </row>
     <row r="6">
@@ -2908,22 +3176,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.698484</v>
+        <v>0.317277</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.707616</v>
+        <v>0.329918</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.716408</v>
+        <v>0.343454</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.724815</v>
+        <v>0.357665</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.72904</v>
+        <v>0.369676</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.182388</v>
+        <v>0.366559</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.174693</v>
       </c>
     </row>
     <row r="7">
@@ -2931,22 +3202,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6793630000000001</v>
+        <v>0.294672</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.692587</v>
+        <v>0.310138</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.705593</v>
+        <v>0.327081</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.718198</v>
+        <v>0.346232</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.728581</v>
+        <v>0.365864</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.182403</v>
+        <v>0.370109</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.174689</v>
       </c>
     </row>
     <row r="8">
@@ -2954,22 +3228,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.660434</v>
+        <v>0.274579</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.677283</v>
+        <v>0.292322</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.694479</v>
+        <v>0.312242</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.7111769999999999</v>
+        <v>0.335182</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.726436</v>
+        <v>0.360639</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.182386</v>
+        <v>0.370714</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.174695</v>
       </c>
     </row>
     <row r="9">
@@ -2977,22 +3254,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.64097</v>
+        <v>0.257385</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.662505</v>
+        <v>0.276269</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.6832780000000001</v>
+        <v>0.298588</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.703989</v>
+        <v>0.324582</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.723368</v>
+        <v>0.354907</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.182387</v>
+        <v>0.369421</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.174692</v>
       </c>
     </row>
     <row r="10">
@@ -3000,22 +3280,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.622152</v>
+        <v>0.242063</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6469510000000001</v>
+        <v>0.262194</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671573</v>
+        <v>0.28587</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.696204</v>
+        <v>0.314433</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.719983</v>
+        <v>0.349044</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.182385</v>
+        <v>0.367298</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.174691</v>
       </c>
     </row>
     <row r="11">
@@ -3023,22 +3306,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.604131</v>
+        <v>0.228299</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.631347</v>
+        <v>0.249336</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.659758</v>
+        <v>0.274394</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.68865</v>
+        <v>0.305111</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.716566</v>
+        <v>0.343325</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.182391</v>
+        <v>0.36477</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.174687</v>
       </c>
     </row>
   </sheetData>
@@ -3067,7 +3353,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -3101,22 +3387,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.51635</v>
+        <v>0.721296</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.516308</v>
+        <v>0.720206</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.515298</v>
+        <v>0.716857</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.511908</v>
+        <v>0.707013</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.499114</v>
+        <v>0.672125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.177993</v>
+        <v>0.182393</v>
       </c>
     </row>
     <row r="5">
@@ -3124,22 +3410,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.509284</v>
+        <v>0.716266</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.512656</v>
+        <v>0.721016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.515756</v>
+        <v>0.725425</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.518181</v>
+        <v>0.728177</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.517415</v>
+        <v>0.723059</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182389</v>
       </c>
     </row>
     <row r="6">
@@ -3147,22 +3433,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.497442</v>
+        <v>0.698484</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.5034380000000001</v>
+        <v>0.707616</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.509286</v>
+        <v>0.716408</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.514854</v>
+        <v>0.724815</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.51884</v>
+        <v>0.72904</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182388</v>
       </c>
     </row>
     <row r="7">
@@ -3170,22 +3456,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.485185</v>
+        <v>0.6793630000000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.493792</v>
+        <v>0.692587</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.502116</v>
+        <v>0.705593</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.510412</v>
+        <v>0.718198</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.517763</v>
+        <v>0.728581</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.177988</v>
+        <v>0.182403</v>
       </c>
     </row>
     <row r="8">
@@ -3193,22 +3479,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.472241</v>
+        <v>0.660434</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.483754</v>
+        <v>0.677283</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.494866</v>
+        <v>0.694479</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.505745</v>
+        <v>0.7111769999999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.515954</v>
+        <v>0.726436</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182386</v>
       </c>
     </row>
     <row r="9">
@@ -3216,22 +3502,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.459365</v>
+        <v>0.64097</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.473397</v>
+        <v>0.662505</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.487421</v>
+        <v>0.6832780000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.50093</v>
+        <v>0.703989</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.513819</v>
+        <v>0.723368</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182387</v>
       </c>
     </row>
     <row r="10">
@@ -3239,22 +3525,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.446312</v>
+        <v>0.622152</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.463127</v>
+        <v>0.6469510000000001</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.479721</v>
+        <v>0.671573</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.495954</v>
+        <v>0.696204</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.511526</v>
+        <v>0.719983</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182385</v>
       </c>
     </row>
     <row r="11">
@@ -3262,22 +3548,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.433206</v>
+        <v>0.604131</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.452681</v>
+        <v>0.631347</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.472072</v>
+        <v>0.659758</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.491045</v>
+        <v>0.68865</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.509188</v>
+        <v>0.716566</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.177987</v>
+        <v>0.182391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ideal all-n=1.8 Al-electrode results to raw-data spreadsheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ideal_n1.8_ITO50" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="n1.80_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="n1.51_ETLHTL500" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="n1.80_t500_ITO50" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="n1.51_t500_ITO50" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="n1.80_ETLHTL500_Al" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="n1.51_ETLHTL500_Al" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="n1.80_ETLHTL80" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="n1.51_ETLHTL80" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="n1.51_ETLHTL150" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="n1.51_ETLHTL200" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ideal_n1.8_ITO50_Al" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="n1.80_ETLHTL500" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="n1.51_ETLHTL500" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="n1.80_t500_ITO50" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.51_t500_ITO50" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="n1.80_ETLHTL500_Al" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="n1.51_ETLHTL500_Al" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="n1.80_ETLHTL80" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="n1.51_ETLHTL80" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="n1.51_ETLHTL150" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="n1.51_ETLHTL200" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,180 +566,198 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL500</t>
+          <t>ideal_n1.8_ITO50_Al</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>IDEAL: all organics n=1.8 lossless, n_sub=n_SL=1.80, ETL/HTL 500 nm, Al electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.2036</v>
+        <v>0.1528</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.8845</v>
+        <v>0.9016</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL500</t>
+          <t>n1.80_ETLHTL500</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.2126</v>
+        <v>0.2036</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.5649</v>
+        <v>0.8845</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL500_Al</t>
+          <t>n1.51_ETLHTL500</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.1778</v>
+        <v>0.2126</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.7775</v>
+        <v>0.5649</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL500_Al</t>
+          <t>n1.80_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.1794</v>
+        <v>0.1778</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.4801</v>
+        <v>0.7775</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>n1.80_t500_ITO50</t>
+          <t>n1.51_ETLHTL500_Al</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.205</v>
+        <v>0.1794</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.8902</v>
+        <v>0.4801</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>n1.51_t500_ITO50</t>
+          <t>n1.80_t500_ITO50</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.222</v>
+        <v>0.205</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.5802</v>
+        <v>0.8902</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL80</t>
+          <t>n1.51_t500_ITO50</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.1854</v>
+        <v>0.222</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.5802</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL80</t>
+          <t>n1.80_ETLHTL80</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.1854</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.5525</v>
+        <v>0.8097</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL150</t>
+          <t>n1.51_ETLHTL80</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.1311</v>
+        <v>0.1865</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.5525</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>n1.51_ETLHTL150</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>0.1311</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>0.4005</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>n1.51_ETLHTL200</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C20" s="2" t="n">
         <v>0.3347</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D20" s="2" t="n">
         <v>0.5671</v>
       </c>
     </row>
@@ -768,7 +787,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -802,22 +821,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.51635</v>
+        <v>0.721296</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.516308</v>
+        <v>0.720206</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.515298</v>
+        <v>0.716857</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.511908</v>
+        <v>0.707013</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.499114</v>
+        <v>0.672125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.177993</v>
+        <v>0.182393</v>
       </c>
     </row>
     <row r="5">
@@ -825,22 +844,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.509284</v>
+        <v>0.716266</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.512656</v>
+        <v>0.721016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.515756</v>
+        <v>0.725425</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.518181</v>
+        <v>0.728177</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.517415</v>
+        <v>0.723059</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182389</v>
       </c>
     </row>
     <row r="6">
@@ -848,22 +867,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.497442</v>
+        <v>0.698484</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.5034380000000001</v>
+        <v>0.707616</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.509286</v>
+        <v>0.716408</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.514854</v>
+        <v>0.724815</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.51884</v>
+        <v>0.72904</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182388</v>
       </c>
     </row>
     <row r="7">
@@ -871,22 +890,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.485185</v>
+        <v>0.6793630000000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.493792</v>
+        <v>0.692587</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.502116</v>
+        <v>0.705593</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.510412</v>
+        <v>0.718198</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.517763</v>
+        <v>0.728581</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.177988</v>
+        <v>0.182403</v>
       </c>
     </row>
     <row r="8">
@@ -894,22 +913,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.472241</v>
+        <v>0.660434</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.483754</v>
+        <v>0.677283</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.494866</v>
+        <v>0.694479</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.505745</v>
+        <v>0.7111769999999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.515954</v>
+        <v>0.726436</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182386</v>
       </c>
     </row>
     <row r="9">
@@ -917,22 +936,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.459365</v>
+        <v>0.64097</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.473397</v>
+        <v>0.662505</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.487421</v>
+        <v>0.6832780000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.50093</v>
+        <v>0.703989</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.513819</v>
+        <v>0.723368</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182387</v>
       </c>
     </row>
     <row r="10">
@@ -940,22 +959,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.446312</v>
+        <v>0.622152</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.463127</v>
+        <v>0.6469510000000001</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.479721</v>
+        <v>0.671573</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.495954</v>
+        <v>0.696204</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.511526</v>
+        <v>0.719983</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182385</v>
       </c>
     </row>
     <row r="11">
@@ -963,22 +982,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.433206</v>
+        <v>0.604131</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.452681</v>
+        <v>0.631347</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.472072</v>
+        <v>0.659758</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.491045</v>
+        <v>0.68865</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.509188</v>
+        <v>0.716566</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.177987</v>
+        <v>0.182391</v>
       </c>
     </row>
   </sheetData>
@@ -1007,7 +1026,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -1041,22 +1060,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.375381</v>
+        <v>0.51635</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.375408</v>
+        <v>0.516308</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.374819</v>
+        <v>0.515298</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.372681</v>
+        <v>0.511908</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.364118</v>
+        <v>0.499114</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.128306</v>
+        <v>0.177993</v>
       </c>
     </row>
     <row r="5">
@@ -1064,22 +1083,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.369639</v>
+        <v>0.509284</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.371995</v>
+        <v>0.512656</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.374193</v>
+        <v>0.515756</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.376003</v>
+        <v>0.518181</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.375864</v>
+        <v>0.517415</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.128304</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="6">
@@ -1087,22 +1106,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.361244</v>
+        <v>0.497442</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.365423</v>
+        <v>0.5034380000000001</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.369509</v>
+        <v>0.509286</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.373419</v>
+        <v>0.514854</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.376431</v>
+        <v>0.51884</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="7">
@@ -1110,22 +1129,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.352561</v>
+        <v>0.485185</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.358622</v>
+        <v>0.493792</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.364454</v>
+        <v>0.502116</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.370239</v>
+        <v>0.510412</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.375481</v>
+        <v>0.517763</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177988</v>
       </c>
     </row>
     <row r="8">
@@ -1133,22 +1152,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.343355</v>
+        <v>0.472241</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.351511</v>
+        <v>0.483754</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.359337</v>
+        <v>0.494866</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.366944</v>
+        <v>0.505745</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.374115</v>
+        <v>0.515954</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="9">
@@ -1156,22 +1175,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.334158</v>
+        <v>0.459365</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.344156</v>
+        <v>0.473397</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.354078</v>
+        <v>0.487421</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.363558</v>
+        <v>0.50093</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.372577</v>
+        <v>0.513819</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="10">
@@ -1179,22 +1198,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.324795</v>
+        <v>0.446312</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.336824</v>
+        <v>0.463127</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.348606</v>
+        <v>0.479721</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.360058</v>
+        <v>0.495954</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.370937</v>
+        <v>0.511526</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="11">
@@ -1202,22 +1221,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.315368</v>
+        <v>0.433206</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.329339</v>
+        <v>0.452681</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.343169</v>
+        <v>0.472072</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.356587</v>
+        <v>0.491045</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.369291</v>
+        <v>0.509188</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177987</v>
       </c>
     </row>
   </sheetData>
@@ -1226,6 +1245,245 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.375381</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.375408</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.374819</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.372681</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.364118</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.128306</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.369639</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.371995</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.374193</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.376003</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.375864</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.128304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.361244</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.365423</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.369509</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.373419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.376431</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.352561</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.358622</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.364454</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.370239</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.375481</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.343355</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.351511</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.359337</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.366944</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.374115</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.334158</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.344156</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.354078</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.363558</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.372577</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.324795</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.336824</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.348606</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.360058</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.370937</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.315368</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.329339</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.343169</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.356587</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.369291</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1747,12 +2005,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>EQE (absolute), IDEAL: all organics n=1.8 lossless, n_sub=n_SL=1.80, ETL/HTL 500 nm, Al electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -1789,25 +2048,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.802346</v>
+        <v>0.590499</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.8015099999999999</v>
+        <v>0.587293</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.798539</v>
+        <v>0.579099</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.789211</v>
+        <v>0.557899</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.753881</v>
+        <v>0.498615</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.679825</v>
+        <v>0.418265</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.206945</v>
+        <v>0.154125</v>
       </c>
     </row>
     <row r="5">
@@ -1815,25 +2074,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.795335</v>
+        <v>0.576744</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.800245</v>
+        <v>0.587241</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.804915</v>
+        <v>0.597066</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.808075</v>
+        <v>0.603104</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.804253</v>
+        <v>0.589916</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.784639</v>
+        <v>0.546369</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.206942</v>
+        <v>0.15412</v>
       </c>
     </row>
     <row r="6">
@@ -1841,25 +2100,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.77694</v>
+        <v>0.540149</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.786347</v>
+        <v>0.55792</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.795369</v>
+        <v>0.576162</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.804036</v>
+        <v>0.594786</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.809096</v>
+        <v>0.604203</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.80163</v>
+        <v>0.5825399999999999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.206943</v>
+        <v>0.15412</v>
       </c>
     </row>
     <row r="7">
@@ -1867,25 +2126,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.756964</v>
+        <v>0.506341</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.770733</v>
+        <v>0.5286999999999999</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.784267</v>
+        <v>0.553409</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.797227</v>
+        <v>0.579542</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.808132</v>
+        <v>0.603278</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.807364</v>
+        <v>0.59768</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.206948</v>
+        <v>0.154135</v>
       </c>
     </row>
     <row r="8">
@@ -1893,25 +2152,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.736989</v>
+        <v>0.477016</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.754758</v>
+        <v>0.502593</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.7727349999999999</v>
+        <v>0.53191</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.790002</v>
+        <v>0.564398</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.805727</v>
+        <v>0.5981</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.809157</v>
+        <v>0.603477</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.20694</v>
+        <v>0.154113</v>
       </c>
     </row>
     <row r="9">
@@ -1919,25 +2178,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.716166</v>
+        <v>0.449873</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.739159</v>
+        <v>0.479596</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.761058</v>
+        <v>0.51212</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.782603</v>
+        <v>0.5494599999999999</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.80248</v>
+        <v>0.590934</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.809593</v>
+        <v>0.605517</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.20694</v>
+        <v>0.154114</v>
       </c>
     </row>
     <row r="10">
@@ -1945,25 +2204,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.695902</v>
+        <v>0.42611</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.7226089999999999</v>
+        <v>0.457585</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.7487819999999999</v>
+        <v>0.492999</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.774516</v>
+        <v>0.534572</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.798996</v>
+        <v>0.582961</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.808812</v>
+        <v>0.60431</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.206939</v>
+        <v>0.15411</v>
       </c>
     </row>
     <row r="11">
@@ -1971,25 +2230,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.676357</v>
+        <v>0.405167</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.705797</v>
+        <v>0.437152</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.736194</v>
+        <v>0.475265</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.766665</v>
+        <v>0.520869</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.7955179999999999</v>
+        <v>0.575473</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.807827</v>
+        <v>0.602531</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.206943</v>
+        <v>0.154122</v>
       </c>
     </row>
   </sheetData>
@@ -2013,13 +2272,12 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
     </row>
@@ -2056,25 +2314,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.530174</v>
+        <v>0.802346</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.530294</v>
+        <v>0.8015099999999999</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.529574</v>
+        <v>0.798539</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.526768</v>
+        <v>0.789211</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.515456</v>
+        <v>0.753881</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.489715</v>
+        <v>0.679825</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.206753</v>
+        <v>0.206945</v>
       </c>
     </row>
     <row r="5">
@@ -2082,25 +2340,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.522313</v>
+        <v>0.795335</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.525689</v>
+        <v>0.800245</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.528843</v>
+        <v>0.804915</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.531454</v>
+        <v>0.808075</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.531369</v>
+        <v>0.804253</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5251749999999999</v>
+        <v>0.784639</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.206942</v>
       </c>
     </row>
     <row r="6">
@@ -2108,25 +2366,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.510482</v>
+        <v>0.77694</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.516444</v>
+        <v>0.786347</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.522269</v>
+        <v>0.795369</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.527867</v>
+        <v>0.804036</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.532183</v>
+        <v>0.809096</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.530655</v>
+        <v>0.80163</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.206943</v>
       </c>
     </row>
     <row r="7">
@@ -2134,25 +2392,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.498234</v>
+        <v>0.756964</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.506833</v>
+        <v>0.770733</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.515134</v>
+        <v>0.784267</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.523386</v>
+        <v>0.797227</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.530869</v>
+        <v>0.808132</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.532184</v>
+        <v>0.807364</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.206948</v>
       </c>
     </row>
     <row r="8">
@@ -2160,25 +2418,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.485254</v>
+        <v>0.736989</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.496809</v>
+        <v>0.754758</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.507911</v>
+        <v>0.7727349999999999</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.51874</v>
+        <v>0.790002</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.528961</v>
+        <v>0.805727</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.532516</v>
+        <v>0.809157</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.206749</v>
+        <v>0.20694</v>
       </c>
     </row>
     <row r="9">
@@ -2186,25 +2444,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.472283</v>
+        <v>0.716166</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.486424</v>
+        <v>0.739159</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.500487</v>
+        <v>0.761058</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.513952</v>
+        <v>0.782603</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.526794</v>
+        <v>0.80248</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.5321050000000001</v>
+        <v>0.809593</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.20694</v>
       </c>
     </row>
     <row r="10">
@@ -2212,25 +2470,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.459081</v>
+        <v>0.695902</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.476091</v>
+        <v>0.7226089999999999</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.492779</v>
+        <v>0.7487819999999999</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.509009</v>
+        <v>0.774516</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.524493</v>
+        <v>0.798996</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.531368</v>
+        <v>0.808812</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.206748</v>
+        <v>0.206939</v>
       </c>
     </row>
     <row r="11">
@@ -2238,25 +2496,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.445793</v>
+        <v>0.676357</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.465539</v>
+        <v>0.705797</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.4851</v>
+        <v>0.736194</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.504113</v>
+        <v>0.766665</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.522168</v>
+        <v>0.7955179999999999</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.53046</v>
+        <v>0.807827</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.206747</v>
+        <v>0.206943</v>
       </c>
     </row>
   </sheetData>
@@ -2286,7 +2544,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
     </row>
@@ -2323,25 +2581,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.824137</v>
+        <v>0.530174</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.823284</v>
+        <v>0.530294</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.820526</v>
+        <v>0.529574</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.811936</v>
+        <v>0.526768</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.778237</v>
+        <v>0.515456</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.70441</v>
+        <v>0.489715</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.207041</v>
+        <v>0.206753</v>
       </c>
     </row>
     <row r="5">
@@ -2349,25 +2607,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.818106</v>
+        <v>0.522313</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.82236</v>
+        <v>0.525689</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.826344</v>
+        <v>0.528843</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.829004</v>
+        <v>0.531454</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.825467</v>
+        <v>0.531369</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.807518</v>
+        <v>0.5251749999999999</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.207039</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="6">
@@ -2375,25 +2633,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.801698</v>
+        <v>0.510482</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.810121</v>
+        <v>0.516444</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.818107</v>
+        <v>0.522269</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.82559</v>
+        <v>0.527867</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.829821</v>
+        <v>0.532183</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.823088</v>
+        <v>0.530655</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.207039</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="7">
@@ -2401,25 +2659,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.783354</v>
+        <v>0.498234</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.796052</v>
+        <v>0.506833</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.808265</v>
+        <v>0.515134</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.819679</v>
+        <v>0.523386</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.829047</v>
+        <v>0.530869</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.828209</v>
+        <v>0.532184</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.207043</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="8">
@@ -2427,25 +2685,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.764553</v>
+        <v>0.485254</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.7812829999999999</v>
+        <v>0.496809</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.797841</v>
+        <v>0.507911</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.813349</v>
+        <v>0.51874</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.8270110000000001</v>
+        <v>0.528961</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.829836</v>
+        <v>0.532516</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.207037</v>
+        <v>0.206749</v>
       </c>
     </row>
     <row r="9">
@@ -2453,25 +2711,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.744617</v>
+        <v>0.472283</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.7665960000000001</v>
+        <v>0.486424</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.787125</v>
+        <v>0.500487</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.806735</v>
+        <v>0.513952</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.824228</v>
+        <v>0.526794</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.830226</v>
+        <v>0.5321050000000001</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.207037</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="10">
@@ -2479,25 +2737,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.724892</v>
+        <v>0.459081</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.750803</v>
+        <v>0.476091</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.775667</v>
+        <v>0.492779</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.799481</v>
+        <v>0.509009</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.82123</v>
+        <v>0.524493</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.829608</v>
+        <v>0.531368</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.207036</v>
+        <v>0.206748</v>
       </c>
     </row>
     <row r="11">
@@ -2505,25 +2763,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.705694</v>
+        <v>0.445793</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.73454</v>
+        <v>0.465539</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.763796</v>
+        <v>0.4851</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.7923</v>
+        <v>0.504113</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.818198</v>
+        <v>0.522168</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.828788</v>
+        <v>0.53046</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.20704</v>
+        <v>0.206747</v>
       </c>
     </row>
   </sheetData>
@@ -2553,7 +2811,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -2590,25 +2848,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.55288</v>
+        <v>0.824137</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.552984</v>
+        <v>0.823284</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.552415</v>
+        <v>0.820526</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.5501470000000001</v>
+        <v>0.811936</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.540554</v>
+        <v>0.778237</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.516624</v>
+        <v>0.70441</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.216258</v>
+        <v>0.207041</v>
       </c>
     </row>
     <row r="5">
@@ -2616,25 +2874,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.546467</v>
+        <v>0.818106</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.549218</v>
+        <v>0.82236</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.551769</v>
+        <v>0.826344</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.553877</v>
+        <v>0.829004</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.5538459999999999</v>
+        <v>0.825467</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5488420000000001</v>
+        <v>0.807518</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="6">
@@ -2642,25 +2900,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.5365799999999999</v>
+        <v>0.801698</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.541612</v>
+        <v>0.810121</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.546428</v>
+        <v>0.818107</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.550978</v>
+        <v>0.82559</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.554465</v>
+        <v>0.829821</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.553283</v>
+        <v>0.823088</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207039</v>
       </c>
     </row>
     <row r="7">
@@ -2668,25 +2926,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.525908</v>
+        <v>0.783354</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.533448</v>
+        <v>0.796052</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.540516</v>
+        <v>0.808265</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.547341</v>
+        <v>0.819679</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.553399</v>
+        <v>0.829047</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.55449</v>
+        <v>0.828209</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207043</v>
       </c>
     </row>
     <row r="8">
@@ -2694,25 +2952,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.514146</v>
+        <v>0.764553</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.524638</v>
+        <v>0.7812829999999999</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.534377</v>
+        <v>0.797841</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.543524</v>
+        <v>0.813349</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.551862</v>
+        <v>0.8270110000000001</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.554735</v>
+        <v>0.829836</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.216255</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="9">
@@ -2720,25 +2978,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.502013</v>
+        <v>0.744617</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.515224</v>
+        <v>0.7665960000000001</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.527905</v>
+        <v>0.787125</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.539524</v>
+        <v>0.806735</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.550112</v>
+        <v>0.824228</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.554397</v>
+        <v>0.830226</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207037</v>
       </c>
     </row>
     <row r="10">
@@ -2746,25 +3004,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.489356</v>
+        <v>0.724892</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.505612</v>
+        <v>0.750803</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.52102</v>
+        <v>0.775667</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.535322</v>
+        <v>0.799481</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.548245</v>
+        <v>0.82123</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.553799</v>
+        <v>0.829608</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.216254</v>
+        <v>0.207036</v>
       </c>
     </row>
     <row r="11">
@@ -2772,25 +3030,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.476366</v>
+        <v>0.705694</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.495584</v>
+        <v>0.73454</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.514006</v>
+        <v>0.763796</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.531089</v>
+        <v>0.7923</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.5463479999999999</v>
+        <v>0.818198</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.553071</v>
+        <v>0.828788</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.216253</v>
+        <v>0.20704</v>
       </c>
     </row>
   </sheetData>
@@ -2820,7 +3078,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL/HTL 500 nm, Ag electrode, ITO 50 nm</t>
         </is>
       </c>
     </row>
@@ -2857,25 +3115,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.527973</v>
+        <v>0.55288</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.527058</v>
+        <v>0.552984</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.522398</v>
+        <v>0.552415</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.508132</v>
+        <v>0.5501470000000001</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.464831</v>
+        <v>0.540554</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.401885</v>
+        <v>0.516624</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.176671</v>
+        <v>0.216258</v>
       </c>
     </row>
     <row r="5">
@@ -2883,25 +3141,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.513765</v>
+        <v>0.546467</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.523353</v>
+        <v>0.549218</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.533013</v>
+        <v>0.551769</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.539902</v>
+        <v>0.553877</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.53354</v>
+        <v>0.5538459999999999</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.5025810000000001</v>
+        <v>0.5488420000000001</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.176663</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="6">
@@ -2909,25 +3167,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.481836</v>
+        <v>0.5365799999999999</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.497634</v>
+        <v>0.541612</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.5140169999999999</v>
+        <v>0.546428</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.531281</v>
+        <v>0.550978</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.542503</v>
+        <v>0.554465</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.529126</v>
+        <v>0.553283</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.176665</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="7">
@@ -2935,25 +3193,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.452262</v>
+        <v>0.525908</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.472202</v>
+        <v>0.533448</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.494101</v>
+        <v>0.540516</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.517697</v>
+        <v>0.547341</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5401</v>
+        <v>0.553399</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.539558</v>
+        <v>0.55449</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.176684</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="8">
@@ -2961,25 +3219,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.426585</v>
+        <v>0.514146</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.4493</v>
+        <v>0.524638</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.475345</v>
+        <v>0.534377</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.504194</v>
+        <v>0.543524</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.534932</v>
+        <v>0.551862</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.5428269999999999</v>
+        <v>0.554735</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.176655</v>
+        <v>0.216255</v>
       </c>
     </row>
     <row r="9">
@@ -2987,25 +3245,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.402791</v>
+        <v>0.502013</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.429294</v>
+        <v>0.515224</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.458065</v>
+        <v>0.527905</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.491371</v>
+        <v>0.539524</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.528176</v>
+        <v>0.550112</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.5435759999999999</v>
+        <v>0.554397</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.176657</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="10">
@@ -3013,25 +3271,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.381897</v>
+        <v>0.489356</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.409937</v>
+        <v>0.505612</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.441454</v>
+        <v>0.52102</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.478134</v>
+        <v>0.535322</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.521226</v>
+        <v>0.548245</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.541695</v>
+        <v>0.553799</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.176651</v>
+        <v>0.216254</v>
       </c>
     </row>
     <row r="11">
@@ -3039,25 +3297,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.363437</v>
+        <v>0.476366</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.391913</v>
+        <v>0.495584</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.425692</v>
+        <v>0.514006</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.466244</v>
+        <v>0.531089</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.514435</v>
+        <v>0.5463479999999999</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.53949</v>
+        <v>0.553071</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.176667</v>
+        <v>0.216253</v>
       </c>
     </row>
   </sheetData>
@@ -3087,7 +3345,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -3124,25 +3382,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.364003</v>
+        <v>0.527973</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.364627</v>
+        <v>0.527058</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.363276</v>
+        <v>0.522398</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.357336</v>
+        <v>0.508132</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.336668</v>
+        <v>0.464831</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.305292</v>
+        <v>0.401885</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.174709</v>
+        <v>0.176671</v>
       </c>
     </row>
     <row r="5">
@@ -3150,25 +3408,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.34348</v>
+        <v>0.513765</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.351908</v>
+        <v>0.523353</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.360201</v>
+        <v>0.533013</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.367467</v>
+        <v>0.539902</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.368065</v>
+        <v>0.53354</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.354522</v>
+        <v>0.5025810000000001</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.174696</v>
+        <v>0.176663</v>
       </c>
     </row>
     <row r="6">
@@ -3176,25 +3434,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.317277</v>
+        <v>0.481836</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.329918</v>
+        <v>0.497634</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.343454</v>
+        <v>0.5140169999999999</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.357665</v>
+        <v>0.531281</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.369676</v>
+        <v>0.542503</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.366559</v>
+        <v>0.529126</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.174693</v>
+        <v>0.176665</v>
       </c>
     </row>
     <row r="7">
@@ -3202,25 +3460,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.294672</v>
+        <v>0.452262</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.310138</v>
+        <v>0.472202</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.327081</v>
+        <v>0.494101</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.346232</v>
+        <v>0.517697</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.365864</v>
+        <v>0.5401</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.370109</v>
+        <v>0.539558</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.174689</v>
+        <v>0.176684</v>
       </c>
     </row>
     <row r="8">
@@ -3228,25 +3486,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.274579</v>
+        <v>0.426585</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.292322</v>
+        <v>0.4493</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.312242</v>
+        <v>0.475345</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.335182</v>
+        <v>0.504194</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.360639</v>
+        <v>0.534932</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.370714</v>
+        <v>0.5428269999999999</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.174695</v>
+        <v>0.176655</v>
       </c>
     </row>
     <row r="9">
@@ -3254,25 +3512,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.257385</v>
+        <v>0.402791</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.276269</v>
+        <v>0.429294</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.298588</v>
+        <v>0.458065</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.324582</v>
+        <v>0.491371</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.354907</v>
+        <v>0.528176</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.369421</v>
+        <v>0.5435759999999999</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.174692</v>
+        <v>0.176657</v>
       </c>
     </row>
     <row r="10">
@@ -3280,25 +3538,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.242063</v>
+        <v>0.381897</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.262194</v>
+        <v>0.409937</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.28587</v>
+        <v>0.441454</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.314433</v>
+        <v>0.478134</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.349044</v>
+        <v>0.521226</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.367298</v>
+        <v>0.541695</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.174691</v>
+        <v>0.176651</v>
       </c>
     </row>
     <row r="11">
@@ -3306,25 +3564,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.228299</v>
+        <v>0.363437</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.249336</v>
+        <v>0.391913</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.274394</v>
+        <v>0.425692</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.305111</v>
+        <v>0.466244</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.343325</v>
+        <v>0.514435</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.36477</v>
+        <v>0.53949</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.174687</v>
+        <v>0.176667</v>
       </c>
     </row>
   </sheetData>
@@ -3338,7 +3596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3348,12 +3606,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3, Al bottom electrode</t>
         </is>
       </c>
     </row>
@@ -3379,6 +3638,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3387,22 +3649,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.721296</v>
+        <v>0.364003</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.720206</v>
+        <v>0.364627</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.716857</v>
+        <v>0.363276</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.707013</v>
+        <v>0.357336</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.672125</v>
+        <v>0.336668</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.182393</v>
+        <v>0.305292</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.174709</v>
       </c>
     </row>
     <row r="5">
@@ -3410,22 +3675,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.716266</v>
+        <v>0.34348</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.721016</v>
+        <v>0.351908</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.725425</v>
+        <v>0.360201</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.728177</v>
+        <v>0.367467</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.723059</v>
+        <v>0.368065</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.182389</v>
+        <v>0.354522</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.174696</v>
       </c>
     </row>
     <row r="6">
@@ -3433,22 +3701,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.698484</v>
+        <v>0.317277</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.707616</v>
+        <v>0.329918</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.716408</v>
+        <v>0.343454</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.724815</v>
+        <v>0.357665</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.72904</v>
+        <v>0.369676</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.182388</v>
+        <v>0.366559</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.174693</v>
       </c>
     </row>
     <row r="7">
@@ -3456,22 +3727,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6793630000000001</v>
+        <v>0.294672</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.692587</v>
+        <v>0.310138</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.705593</v>
+        <v>0.327081</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.718198</v>
+        <v>0.346232</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.728581</v>
+        <v>0.365864</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.182403</v>
+        <v>0.370109</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.174689</v>
       </c>
     </row>
     <row r="8">
@@ -3479,22 +3753,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.660434</v>
+        <v>0.274579</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.677283</v>
+        <v>0.292322</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.694479</v>
+        <v>0.312242</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.7111769999999999</v>
+        <v>0.335182</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.726436</v>
+        <v>0.360639</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.182386</v>
+        <v>0.370714</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.174695</v>
       </c>
     </row>
     <row r="9">
@@ -3502,22 +3779,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.64097</v>
+        <v>0.257385</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.662505</v>
+        <v>0.276269</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.6832780000000001</v>
+        <v>0.298588</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.703989</v>
+        <v>0.324582</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.723368</v>
+        <v>0.354907</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.182387</v>
+        <v>0.369421</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.174692</v>
       </c>
     </row>
     <row r="10">
@@ -3525,22 +3805,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.622152</v>
+        <v>0.242063</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6469510000000001</v>
+        <v>0.262194</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671573</v>
+        <v>0.28587</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.696204</v>
+        <v>0.314433</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.719983</v>
+        <v>0.349044</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.182385</v>
+        <v>0.367298</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.174691</v>
       </c>
     </row>
     <row r="11">
@@ -3548,22 +3831,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.604131</v>
+        <v>0.228299</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.631347</v>
+        <v>0.249336</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.659758</v>
+        <v>0.274394</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.68865</v>
+        <v>0.305111</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.716566</v>
+        <v>0.343325</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.182391</v>
+        <v>0.36477</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.174687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>